<commit_message>
add 10 test case
</commit_message>
<xml_diff>
--- a/test-cases/test-cases.xlsx
+++ b/test-cases/test-cases.xlsx
@@ -1,17 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E245D16-4CA1-471C-B2C0-6E19FFB2FF1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="ปรับปรุง Test Case ตามหลักการ W" sheetId="1" r:id="rId5"/>
+    <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="247">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -518,20 +532,255 @@
   </si>
   <si>
     <t>เซิร์ฟเวอร์ทำงานลื่นไหลปกติ</t>
+  </si>
+  <si>
+    <t>TC-021</t>
+  </si>
+  <si>
+    <t>Security - User Enumeration</t>
+  </si>
+  <si>
+    <t>ทดสอบป้องกันการเดาอีเมลผู้ใช้ในระบบจากหน้าลืมรหัสผ่าน</t>
+  </si>
+  <si>
+    <t>ผู้ใช้อยู่ที่หน้า "ลืมรหัสผ่าน" (Forgot Password)</t>
+  </si>
+  <si>
+    <t>Email: notexist@email.com (อีเมลที่ไม่มีจริง)</t>
+  </si>
+  <si>
+    <t>1. ไปหน้าลืมรหัสผ่าน2. ใส่อีเมลที่ไม่มีในระบบ3. กดส่งลิงก์รีเซ็ต</t>
+  </si>
+  <si>
+    <t>1. ระบบแสดงข้อความกลางๆ เช่น "หากมีอีเมลนี้ในระบบ เราได้ส่งลิงก์ไปให้แล้ว"2. ต้องไม่แสดงข้อความว่า "ไม่พบอีเมลนี้"</t>
+  </si>
+  <si>
+    <t>ไม่มีอีเมลถูกส่งออกไป</t>
+  </si>
+  <si>
+    <t>TC-022</t>
+  </si>
+  <si>
+    <t>Security - Mass Assignment Profile</t>
+  </si>
+  <si>
+    <t>ทดสอบป้องกันการแอบอัปเกรดสิทธิ์ตัวเองผ่าน API</t>
+  </si>
+  <si>
+    <t>JSON Body: {"name":"test","role":"admin"}</t>
+  </si>
+  <si>
+    <t>1. ใช้ Postman ส่ง API (PUT) แก้ไขข้อมูลส่วนตัว2. แอบแนบฟิลด์ "role": "admin" เข้าไป</t>
+  </si>
+  <si>
+    <t>1. บันทึกชื่อใหม่สำเร็จ2. ระบบต้องเพิกเฉยต่อฟิลด์ role3. สิทธิ์ยังเป็น User ปกติ</t>
+  </si>
+  <si>
+    <t>ชื่อเปลี่ยน แต่สิทธิ์ยังเหมือนเดิม</t>
+  </si>
+  <si>
+    <t>TC-023</t>
+  </si>
+  <si>
+    <t>Security - API Rate Limiting</t>
+  </si>
+  <si>
+    <t>ทดสอบการป้องกัน DoS / สแปม Request</t>
+  </si>
+  <si>
+    <t>ระบบทำงานปกติ</t>
+  </si>
+  <si>
+    <t>API Endpoint: /api/books (ยิง 100 ครั้งใน 1 วิ)</t>
+  </si>
+  <si>
+    <t>1. ใช้ Postman Runner หรือสคริปต์ยิง API ค้นหาหนังสือรัวๆ 100 ครั้งใน 1 วินาที</t>
+  </si>
+  <si>
+    <t>1. ช่วงแรกโหลดข้อมูลได้2. หลังจากเกิน Limit ระบบบล็อกและตอบกลับ HTTP 429 Too Many Requests</t>
+  </si>
+  <si>
+    <t>ระบบยังทำงานได้ปกติ ไม่ล่ม</t>
+  </si>
+  <si>
+    <t>TC-024</t>
+  </si>
+  <si>
+    <t>Security - Information Exposure</t>
+  </si>
+  <si>
+    <t>ทดสอบว่า Error ไม่หลุดข้อมูล Database ออกมา</t>
+  </si>
+  <si>
+    <t>Book ID = abc (ใส่ตัวอักษรแทนตัวเลข)</t>
+  </si>
+  <si>
+    <t>1. เรียก API ขอดูข้อมูลหนังสือ GET /api/books/abc</t>
+  </si>
+  <si>
+    <t>1. ปฏิเสธ Request2. ตอบ HTTP 400 Bad Request3. ไม่มี Stack Trace หรือ โค้ด SQL โผล่มาที่หน้าจอ</t>
+  </si>
+  <si>
+    <t>ไม่มีข้อมูลรั่วไหล</t>
+  </si>
+  <si>
+    <t>TC-025</t>
+  </si>
+  <si>
+    <t>Security - Path Traversal</t>
+  </si>
+  <si>
+    <t>ทดสอบการแอบดูไฟล์ระบบผ่าน API ดึงรูป</t>
+  </si>
+  <si>
+    <t>มีรูปภาพโปรไฟล์อยู่ในระบบ</t>
+  </si>
+  <si>
+    <t>URL: /images?file=../../../../etc/passwd</t>
+  </si>
+  <si>
+    <t>1. เรียก API ดูรูปภาพ2. แก้ไขพารามิเตอร์ไฟล์ให้เป็น Path ย้อนกลับไปดูไฟล์ระบบ</t>
+  </si>
+  <si>
+    <t>1. ระบบต้องกรอง Path2. ตอบ HTTP 403 Forbidden หรือ 404 Not Found</t>
+  </si>
+  <si>
+    <t>ไม่สามารถเข้าถึงไฟล์ระบบได้</t>
+  </si>
+  <si>
+    <t>TC-026</t>
+  </si>
+  <si>
+    <t>Business Logic - Borrow unavailable</t>
+  </si>
+  <si>
+    <t>ทดสอบลอจิกการยืมหนังสือที่ถูกยืมไปแล้ว (หมดสต็อก)</t>
+  </si>
+  <si>
+    <t>หนังสือ ID: 1 มีสถานะ "ถูกยืมแล้ว" หรือสต็อกเป็น 0</t>
+  </si>
+  <si>
+    <t>Book ID: 1</t>
+  </si>
+  <si>
+    <t>1. ล็อกอินเป็น User ปกติ2. ส่งคำสั่งกดยืมหนังสือ ID 1</t>
+  </si>
+  <si>
+    <t>1. ยืมไม่สำเร็จ2. ระบบแจ้งเตือน "หนังสือเล่มนี้ไม่พร้อมให้บริการ"</t>
+  </si>
+  <si>
+    <t>สต็อกหนังสือไม่ติดลบ</t>
+  </si>
+  <si>
+    <t>TC-027</t>
+  </si>
+  <si>
+    <t>Security - Token reuse after Logout</t>
+  </si>
+  <si>
+    <t>ทดสอบการจัดการ Session ที่ไม่ปลอดภัยหลัง Logout</t>
+  </si>
+  <si>
+    <t>ล็อกอินและเก็บ JWT Token ไว้</t>
+  </si>
+  <si>
+    <t>Token ที่เพิ่งถูกใช้งาน</t>
+  </si>
+  <si>
+    <t>1. ล็อกอินและก็อปปี้ Token ไว้2. กด Logout3. นำ Token เดิมไปยิง API ขอดูโปรไฟล์ผ่าน Postman</t>
+  </si>
+  <si>
+    <t>1. ระบบไม่อนุญาตให้ใช้ Token นั้นอีก2. ตอบ HTTP 401 Unauthorized</t>
+  </si>
+  <si>
+    <t>โทเคนถูกทำลายหรือแบล็คลิสต์</t>
+  </si>
+  <si>
+    <t>TC-028</t>
+  </si>
+  <si>
+    <t>Security - HTTP Method Tampering</t>
+  </si>
+  <si>
+    <t>ทดสอบส่ง Method ผิดประเภทไปที่ API</t>
+  </si>
+  <si>
+    <t>ทราบ Endpoint ของ API</t>
+  </si>
+  <si>
+    <t>ส่ง POST ไปที่ API GET /api/books</t>
+  </si>
+  <si>
+    <t>1. ใช้ Postman ส่ง Request แบบ POST (สร้างข้อมูล) ไปยัง URL ที่รับเฉพาะ GET</t>
+  </si>
+  <si>
+    <t>1. ระบบปฏิเสธคำสั่งทันที2. ตอบกลับด้วย HTTP 405 Method Not Allowed</t>
+  </si>
+  <si>
+    <t>ไม่มีข้อมูลถูกสร้างใหม่</t>
+  </si>
+  <si>
+    <t>TC-029</t>
+  </si>
+  <si>
+    <t>Security - XSS in SVG Upload</t>
+  </si>
+  <si>
+    <t>ทดสอบฝัง XSS ในไฟล์ภาพแบบ SVG</t>
+  </si>
+  <si>
+    <t>ล็อกอินเข้าสู่หน้าแก้ไขโปรไฟล์</t>
+  </si>
+  <si>
+    <t>ไฟล์ xss.svg ที่แอบฝัง &lt;script&gt; ไว้</t>
+  </si>
+  <si>
+    <t>1. อัปโหลดไฟล์รูป .svg อันตราย2. เปิดดูรูปภาพบน Browser</t>
+  </si>
+  <si>
+    <t>1. ระบบปฏิเสธไฟล์ .svg ตั้งแต่แรก หรือ2. ถ้าให้ผ่าน ต้อง Sanitize โค้ดอันตรายออก Script ต้องไม่ทำงาน</t>
+  </si>
+  <si>
+    <t>บัญชีผู้ใช้ยังปลอดภัยจาก XSS</t>
+  </si>
+  <si>
+    <t>TC-030</t>
+  </si>
+  <si>
+    <t>Security - CSRF on Password Change</t>
+  </si>
+  <si>
+    <t>ทดสอบการเปลี่ยนรหัสโดยไม่ส่งตัวป้องกัน CSRF</t>
+  </si>
+  <si>
+    <t>ล็อกอินสำเร็จ</t>
+  </si>
+  <si>
+    <t>Request การเปลี่ยนรหัสที่ไม่มี CSRF Token</t>
+  </si>
+  <si>
+    <t>1. ใช้ Postman จำลองการยิง API เปลี่ยนรหัสผ่าน2. ไม่แนบ CSRF Token ใน Header/Body</t>
+  </si>
+  <si>
+    <t>1. ระบบปฏิเสธคำสั่ง2. ตอบ HTTP 403 Forbidden3. แจ้งเตือน Invalid CSRF Token</t>
+  </si>
+  <si>
+    <t>รหัสผ่านยังคงเป็นรหัสเดิม</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -542,70 +791,37 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF356854"/>
-          <bgColor rgb="FF356854"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <border>
         <left style="thin">
@@ -622,20 +838,48 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="ปรับปรุง Test Case ตามหลักการ W-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="รวม 30 Test Case Design-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -643,26 +887,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:K21" displayName="Security_Test_Cases" name="Security_Test_Cases" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Security_Test_Cases" displayName="Security_Test_Cases" ref="A1:K31">
   <tableColumns count="11">
-    <tableColumn name="Test Case ID" id="1"/>
-    <tableColumn name="Test Case Title" id="2"/>
-    <tableColumn name="Description" id="3"/>
-    <tableColumn name="Priority" id="4"/>
-    <tableColumn name="Preconditions" id="5"/>
-    <tableColumn name="Test Data" id="6"/>
-    <tableColumn name="Test Steps" id="7"/>
-    <tableColumn name="Expected Results" id="8"/>
-    <tableColumn name="Actual Results" id="9"/>
-    <tableColumn name="Status" id="10"/>
-    <tableColumn name="Postconditions" id="11"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Test Case ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Case Title"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Priority"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Preconditions"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Test Data"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Test Steps"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Expected Results"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Actual Results"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Status"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Postconditions"/>
   </tableColumns>
-  <tableStyleInfo name="ปรับปรุง Test Case ตามหลักการ W-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="รวม 30 Test Case Design-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -852,27 +1096,30 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:K31"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="15.0"/>
-    <col customWidth="1" min="2" max="2" width="28.25"/>
-    <col customWidth="1" min="3" max="3" width="35.5"/>
-    <col customWidth="1" min="4" max="4" width="13.88"/>
-    <col customWidth="1" min="5" max="5" width="28.38"/>
-    <col customWidth="1" min="6" max="8" width="37.63"/>
-    <col customWidth="1" min="9" max="9" width="16.13"/>
-    <col customWidth="1" min="11" max="11" width="31.88"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="28.42578125" customWidth="1"/>
+    <col min="6" max="8" width="37.5703125" customWidth="1"/>
+    <col min="9" max="9" width="16.140625" customWidth="1"/>
+    <col min="11" max="11" width="31.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
+    <row r="1" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -907,7 +1154,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -939,7 +1186,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
+    <row r="3" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
@@ -971,7 +1218,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
+    <row r="4" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
@@ -1003,7 +1250,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
+    <row r="5" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>38</v>
       </c>
@@ -1035,7 +1282,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
+    <row r="6" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>46</v>
       </c>
@@ -1067,7 +1314,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
+    <row r="7" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>54</v>
       </c>
@@ -1099,7 +1346,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
+    <row r="8" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>62</v>
       </c>
@@ -1131,7 +1378,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
+    <row r="9" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>70</v>
       </c>
@@ -1163,7 +1410,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
+    <row r="10" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>78</v>
       </c>
@@ -1195,7 +1442,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
+    <row r="11" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>86</v>
       </c>
@@ -1227,7 +1474,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1">
+    <row r="12" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>94</v>
       </c>
@@ -1259,7 +1506,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
+    <row r="13" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>102</v>
       </c>
@@ -1291,7 +1538,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" ht="22.5" customHeight="1">
+    <row r="14" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>110</v>
       </c>
@@ -1323,7 +1570,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="15" ht="22.5" customHeight="1">
+    <row r="15" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>118</v>
       </c>
@@ -1355,7 +1602,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="16" ht="22.5" customHeight="1">
+    <row r="16" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>125</v>
       </c>
@@ -1387,7 +1634,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="17" ht="22.5" customHeight="1">
+    <row r="17" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>132</v>
       </c>
@@ -1419,7 +1666,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="18" ht="22.5" customHeight="1">
+    <row r="18" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>139</v>
       </c>
@@ -1451,7 +1698,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
+    <row r="19" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>147</v>
       </c>
@@ -1483,7 +1730,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="20" ht="22.5" customHeight="1">
+    <row r="20" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>154</v>
       </c>
@@ -1515,7 +1762,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="21" ht="22.5" customHeight="1">
+    <row r="21" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>161</v>
       </c>
@@ -1547,15 +1794,335 @@
         <v>168</v>
       </c>
     </row>
+    <row r="22" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="D2:D21">
-      <formula1>"High,Critical,Medium"</formula1>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D31" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>"High,Critical,Medium,low"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>